<commit_message>
feat: URL Finder - Reset button always visible + no-cache mode
- Reset button visible during running (cancels job first)
- Add --no-cache flag to Python script
- Web UI always uses --no-cache for fresh results
- Prevents cached results when re-running same file
</commit_message>
<xml_diff>
--- a/test_hotels.xlsx
+++ b/test_hotels.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,42 +413,98 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>child_hotel_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>child_hotel_address</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Lotte Hotel Hanoi</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1861</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>54 Lieu Giai, Ba Dinh, Hanoi</t>
+          <t>Elaya Hotel Steinplatte Ehemals Kuhotel by Rilano</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sonnwendstraße 13b</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Sofitel Legend Metropole Hanoi</t>
-        </is>
+      <c r="A3" t="n">
+        <v>1862</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>15 Ngo Quyen, Hoan Kiem, Hanoi</t>
+          <t>Levi Hotel Spa</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Levintie 1590, LEVI PF, Sirkka, Kittila, Lapland, 99130, Finland</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1863</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Residence Cala Liberotto</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Viale Calaliberotto, Orosei, Sardinia, 08028, Italy</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1864</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Barnett Hill - Luxury Hotel</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Blackheath Lane</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1865</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Katerina Hotel</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Naxos island, Ag. Prokopios, Agios Prokopios, South Aegean, 84300, Greece</t>
         </is>
       </c>
     </row>

</xml_diff>